<commit_message>
added subsection level extraction for regulations, need to test with servers
</commit_message>
<xml_diff>
--- a/Pravartiya/data/output_excels/circulars-2026-04/SEBI.xlsx
+++ b/Pravartiya/data/output_excels/circulars-2026-04/SEBI.xlsx
@@ -535,9 +535,9 @@
 Existing Provision of Law:
 Not specifically stated.
 Gist of amendment of that regulation:
-SEBI has issued this circular and modified a one-time relaxation for specified securities, allowing them to be recorded as "non-transferable" by Depositories during applicable lock-in periods. Stock Exchanges, Depositories, Merchant Bankers, and issuers must ensure compliance with this mechanism for pledged shares lock-in.
+The SEBI has issued this circular and amended (Issue of Capital and Disclosure Requirements) Regulations, 2018 to allow for specified securities on which lock-in cannot be created, to be recorded as "non-transferable" by Depositories during the applicable lock-in period. Issuers are required to incorporate suitable provisions in their Articles of Association, issue necessary intimations to concerned lenders/pledges, and make suitable disclosures in offer documents. Stock Exchanges, Depositories, Merchant Bankers, and issuers must ensure compliance with this new mechanism for lock-in of pledged shares.
 Action point for listed entity:
-Stock Exchanges, Depositories, Merchant Bankers, and issuers shall ensure compliance with the mechanism for lock-in of pledged shares as per the amended SEBI (Issue of Capital and Disclosure Requirements) Regulations, 2018.</t>
+Stock Exchanges, Depositories, Merchant Bankers, and issuers shall ensure compliance with the mechanism for lock-in of pledged shares.</t>
         </is>
       </c>
     </row>
@@ -594,11 +594,11 @@
 Regulation Number:
 SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015
 Existing Provision of Law:
-Before the amendment, listed entities that did not comply with Minimum Public Shareholding (MPS) requirements were subject to penal provisions under the SEBI Master Circular dated July 11, 2023 for compliance with the provisions of the SEBI (Listing Obligations and Disclosure Requirements) Regulations, 2015. These penalties included fines, freezing of promoter shareholding, and other consequential actions. The Master Circular also specified a procedure to be followed by recognized stock exchanges and depositories in respect of listed entities not complying with MPS requirements.
+In case a listed entity does not comply with Minimum Public Shareholding (MPS) requirements, as per the SEBI Master Circular dated July 11, 2023, stock exchanges and depositories are required to take penal actions such as levying fines, freezing promoter shareholding, and other consequential actions.
 Gist of amendment of that regulation:
-SEBI has issued this circular and modified a one-time relaxation for listed entities whose due date for Minimum Public Shareholding (MPS) compliance falls between April 1, 2026, and September 30, 2026. Recognized stock exchanges and depositories are advised not to levy fines or freeze promoter shareholding against such entities during this period.
+The SEBI has issued this circular and granted a one-time relaxation from the applicability of penal provisions under the SEBI Master Circular for listed entities whose due date for compliance with Minimum Public Shareholding (MPS) requirements falls during the period from April 1, 2026 to September 30, 2026. Recognized stock exchanges and depositories are advised not to take any penal action against such entities for non-compliance during the said period, and any initiated penal actions may be withdrawn. Stock exchanges have been advised to bring this circular to the notice of listed entities and make necessary amendments to relevant bye-laws, rules, and regulations for its implementation.
 Action point for listed entity:
-Recognized Stock Exchanges and Depositories shall not take any penal action against listed entities whose due date for compliance with Minimum Public Shareholding (MPS) requirements falls during the period from April 1, 2026 to September 30, 2026.</t>
+No specific action point identified.</t>
         </is>
       </c>
     </row>
@@ -655,11 +655,11 @@
 Regulation Number:
 Regulations 44(1) and 59C of SEBI (Issue of Capital and Disclosure Requirements) Regulations, 2018 (ICDR Regulations, 2018)
 Existing Provision of Law:
-In terms of Regulations 44(1) and 59C of SEBI (Issue of Capital and Disclosure Requirements) Regulations, 2018 (ICDR Regulations, 2018), a public issue may be opened within twelve months from the date of issuance of observations by SEBI for regulations 44(1), and within eighteen months for regulations 59C.
+In terms of Regulations 44(1) and 59C of SEBI (Issue of Capital and Disclosure Requirements) Regulations, 2018 (ICDR Regulations, 2018), a public issue may be opened within twelve months and eighteen months respectively from the date of issuance of observations by SEBI.
 Gist of amendment of that regulation:
-SEBI has issued this circular and modified a one-time relaxation for extending the validity of SEBI Observations letters, expiring between April 1, 2026 - September 30, 2026, till September 30, 2026. This applies to all entities proposing to list specified securities and is subject to an undertaking from the Lead Manager confirming compliance with Schedule XVI of the ICDR Regulations while submitting the updated offer document to the Board.
+The SEBI has issued this circular and granted a one-time relaxation to extend the validity of SEBI Observations letters, expiring between April 1, 2026 - September 30, 2026, till September 30, 2026, subject to an undertaking from Lead Manager to the issue confirming compliance with Schedule XVI of the ICDR Regulations while submitting the updated offer document to the Board. This circular comes into force immediately.
 Action point for listed entity:
-Registered Merchant Bankers, Recognized Stock Exchanges and entities proposing to list specified securities shall ensure compliance with Schedule XVI of the ICDR Regulations while submitting the updated offer document to SEBI, extending validity of SEBI Observations letters expiring between April 1, 2026 - September 30, 2026 till September 30, 2026.</t>
+Registered Merchant Bankers and entities who propose to list specified securities shall ensure compliance with Schedule XVI of the ICDR Regulations while submitting the updated offer document to the Board, in case their SEBI Observations letters expire between April 1, 2026 - September 30, 2026.</t>
         </is>
       </c>
     </row>

</xml_diff>